<commit_message>
fix: resolve NameError in build_caption and verify custom Cloudinary folder
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1363,6 +1363,33 @@
         </is>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>scenic</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>DXj4ZZ_jcuR</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>reel</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026-05-12 19:22:55 UTC</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DXj4ZZ_jcuR/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>scenic</t>
         </is>

</xml_diff>